<commit_message>
Add correlations between exposures
</commit_message>
<xml_diff>
--- a/Output/Descriptive_exposure_tables_malf.xlsx
+++ b/Output/Descriptive_exposure_tables_malf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/estela_blanco_uc_cl/Documents/Contaminación_Malformaciones Congénitas/Pollution_Malformation_TEM/Output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_4EBE6243CCEE49D1477B1E9311066B43C4B25038" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4F8935F-98BF-7B40-96A3-670CD3F02682}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_4EBE6243CCEE49D1477B1E9311066B43C4B25038" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E78021E8-B715-BE44-89C0-AB1C08A1E0B5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" firstSheet="2" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full_sample_PM25" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,20 @@
     <sheet name="Malf_card_bin_1_Levo" sheetId="14" r:id="rId14"/>
     <sheet name="Malf_card_bin_1_K" sheetId="15" r:id="rId15"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -3290,11 +3303,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11941,13 +11955,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -11958,7 +11972,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -11969,7 +11983,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -11980,7 +11994,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -11991,7 +12005,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -12002,7 +12016,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -12012,8 +12026,26 @@
       <c r="C6" t="s">
         <v>460</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D6">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="E6">
+        <v>14.27</v>
+      </c>
+      <c r="F6" s="2">
+        <f>E6/2</f>
+        <v>7.1349999999999998</v>
+      </c>
+      <c r="G6" s="2">
+        <f>D6-F6</f>
+        <v>27.164999999999999</v>
+      </c>
+      <c r="H6" s="2">
+        <f>D6+F6</f>
+        <v>41.434999999999995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -12023,8 +12055,26 @@
       <c r="C7" t="s">
         <v>462</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D7">
+        <v>51.7</v>
+      </c>
+      <c r="E7">
+        <v>29.42</v>
+      </c>
+      <c r="F7" s="2">
+        <f>E7/2</f>
+        <v>14.71</v>
+      </c>
+      <c r="G7" s="2">
+        <f>D7-F7</f>
+        <v>36.99</v>
+      </c>
+      <c r="H7" s="2">
+        <f>D7+F7</f>
+        <v>66.41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -12035,7 +12085,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -12046,7 +12096,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -12057,7 +12107,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -12068,7 +12118,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -12079,7 +12129,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -12090,7 +12140,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -12101,7 +12151,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -12112,7 +12162,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>45</v>
       </c>

</xml_diff>